<commit_message>
update: Week 23 complete - add Chun Chieh 16.44km walk, Jeremy 7.38km run; recalculate all cumulative scores accurately
</commit_message>
<xml_diff>
--- a/Reports/Members/Chun Chieh_Activity_Report.xlsx
+++ b/Reports/Members/Chun Chieh_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,6 +506,53 @@
         </is>
       </c>
       <c r="I2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>6/7/2026 17:27:12</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chun Chieh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>16.44</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>25,078</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -554,10 +601,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.92</v>
+        <v>22.36</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>25078</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -624,10 +671,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.92</v>
+        <v>22.36</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>25078</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>

</xml_diff>